<commit_message>
NRF Fixes, Interrupt Fixes, PCB fixes, controller fixes.
</commit_message>
<xml_diff>
--- a/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
+++ b/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e_vadeboncoeur\Documents\PlatformIO\Projects\Hexapod v3\Design\Mechanical Design\Kinematics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D969643-B5E1-4F91-A934-B932115A8C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD79CC9-FD29-43FC-9CF6-10D8D0DE317A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
   </bookViews>
   <sheets>
     <sheet name="X" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="XY" sheetId="3" r:id="rId3"/>
     <sheet name="W" sheetId="4" r:id="rId4"/>
     <sheet name="XYW" sheetId="5" r:id="rId5"/>
+    <sheet name="RC Calculations" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">W!$A$4:$A$10</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="59">
   <si>
     <t>Leg</t>
   </si>
@@ -93,13 +94,156 @@
   <si>
     <t>Wz:</t>
   </si>
+  <si>
+    <t>Constants</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit </t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>PI/6</t>
+  </si>
+  <si>
+    <t>PI/3</t>
+  </si>
+  <si>
+    <t>rad</t>
+  </si>
+  <si>
+    <t>Calculations</t>
+  </si>
+  <si>
+    <t>ADC MAX</t>
+  </si>
+  <si>
+    <t>X ADC Max</t>
+  </si>
+  <si>
+    <t>Y ADC Max</t>
+  </si>
+  <si>
+    <t>V mag min</t>
+  </si>
+  <si>
+    <t>V mag max</t>
+  </si>
+  <si>
+    <t>X ADC Mid</t>
+  </si>
+  <si>
+    <t>Y ADC Mid</t>
+  </si>
+  <si>
+    <t>ADC MIN</t>
+  </si>
+  <si>
+    <t>bits</t>
+  </si>
+  <si>
+    <t>mm/s</t>
+  </si>
+  <si>
+    <t>ADC X</t>
+  </si>
+  <si>
+    <t>ADC Y</t>
+  </si>
+  <si>
+    <t>V map</t>
+  </si>
+  <si>
+    <t>V adc</t>
+  </si>
+  <si>
+    <t>ADC XC</t>
+  </si>
+  <si>
+    <t>ADC YC</t>
+  </si>
+  <si>
+    <t>X ADC Min</t>
+  </si>
+  <si>
+    <t>Y ADC Min</t>
+  </si>
+  <si>
+    <t>Center Shift</t>
+  </si>
+  <si>
+    <t>X ADC MaxS</t>
+  </si>
+  <si>
+    <t>X ADC MinS</t>
+  </si>
+  <si>
+    <t>Y ADC MaxS</t>
+  </si>
+  <si>
+    <t>Y ADC MinS</t>
+  </si>
+  <si>
+    <t>V adc Max</t>
+  </si>
+  <si>
+    <t>V adc Min</t>
+  </si>
+  <si>
+    <t>Theta T1</t>
+  </si>
+  <si>
+    <t>Theta T2</t>
+  </si>
+  <si>
+    <t>Quantized</t>
+  </si>
+  <si>
+    <t>Theta T2D</t>
+  </si>
+  <si>
+    <t>deg</t>
+  </si>
+  <si>
+    <t>vx</t>
+  </si>
+  <si>
+    <t>vy</t>
+  </si>
+  <si>
+    <t>along robot +X</t>
+  </si>
+  <si>
+    <t>along robot +Y</t>
+  </si>
+  <si>
+    <t>V clamp</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -115,7 +259,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -123,12 +267,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8032,4 +8261,440 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E776AA44-A3C8-43E7-96F1-C4D35D29F60B}">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="6"/>
+      <c r="F1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2">
+        <f>PI()/6</f>
+        <v>0.52359877559829882</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="2">
+        <v>4095</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2">
+        <f>PI()/3</f>
+        <v>1.0471975511965976</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4095</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="2">
+        <f>G3-B14</f>
+        <v>2048</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="2">
+        <f>G4-B16</f>
+        <v>953</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1958</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="2">
+        <f>SQRT(G5*G5+G6*G6)</f>
+        <v>2258.8742771566549</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1958</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="2">
+        <f>(G7)*((B21-B20)/(B18-B19))+B20</f>
+        <v>154.41523379000571</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2">
+        <f>B5-B7</f>
+        <v>2137</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="2">
+        <f>IF(G8&gt;B21, B21,G8)</f>
+        <v>140</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="2">
+        <f>B5-B8</f>
+        <v>2137</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="2">
+        <f>ATAN2(G5,G6)</f>
+        <v>0.43553063969993661</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="2">
+        <f>B6-B7</f>
+        <v>-1958</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="2">
+        <f>B4*ROUND(G10/B4, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="2">
+        <f>B6-B8</f>
+        <v>-1958</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="2">
+        <f>DEGREES(G11)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="2">
+        <v>90</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="2">
+        <f>G9*COS(G11)</f>
+        <v>140</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="2">
+        <f>B9-B13</f>
+        <v>2047</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="2">
+        <f>G9*SIN(G11)</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="2">
+        <f>B11-B13</f>
+        <v>-2048</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="2">
+        <f>B14</f>
+        <v>2047</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="2">
+        <f>B15</f>
+        <v>-2048</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="2">
+        <v>2048</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="2">
+        <v>0</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="2">
+        <v>140</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
More ripple gait code.
</commit_message>
<xml_diff>
--- a/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
+++ b/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e_vadeboncoeur\Documents\PlatformIO\Projects\Hexapod v3\Design\Mechanical Design\Kinematics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD79CC9-FD29-43FC-9CF6-10D8D0DE317A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2F866A-B2F8-449B-A2F3-0D24835391C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
   </bookViews>
   <sheets>
     <sheet name="X" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="W" sheetId="4" r:id="rId4"/>
     <sheet name="XYW" sheetId="5" r:id="rId5"/>
     <sheet name="RC Calculations" sheetId="6" r:id="rId6"/>
+    <sheet name="Ripple Phase" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">W!$A$4:$A$10</definedName>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="71">
   <si>
     <t>Leg</t>
   </si>
@@ -229,6 +230,42 @@
   <si>
     <t>test</t>
   </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>Leg 0</t>
+  </si>
+  <si>
+    <t>Leg 1</t>
+  </si>
+  <si>
+    <t>Leg 2</t>
+  </si>
+  <si>
+    <t>Leg 3</t>
+  </si>
+  <si>
+    <t>Leg 4</t>
+  </si>
+  <si>
+    <t>Leg 5</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Cycle Const</t>
+  </si>
+  <si>
+    <t>s_total</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
 </sst>
 </file>
 
@@ -344,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -358,6 +395,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8697,4 +8739,186 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3AFBAB9-467F-4E05-A5CF-E22C3165A618}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="2">
+        <f>1/6</f>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="F3" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <f>$B$5-(ABS(G4-$B$4)*$B$3)</f>
+        <v>1</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <f>$B$5-(ABS(G5-$B$4)*$B$3)</f>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2">
+        <f>$B$5-(ABS(G6-$B$4)*$B$3)</f>
+        <v>0.66666666666666674</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="2">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2">
+        <f>$B$5-(ABS(G7-$B$4)*$B$3)</f>
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="2">
+        <v>4</v>
+      </c>
+      <c r="H8" s="2">
+        <f>$B$5-(ABS(G8-$B$4)*$B$3)</f>
+        <v>0.33333333333333337</v>
+      </c>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5</v>
+      </c>
+      <c r="H9" s="2">
+        <f>$B$5-(ABS(G9-$B$4)*$B$3)</f>
+        <v>0.16666666666666674</v>
+      </c>
+      <c r="I9" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
state, comm, ram, startup changes
</commit_message>
<xml_diff>
--- a/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
+++ b/Design/Mechanical Design/Kinematics/Body Kinematics Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e_vadeboncoeur\Documents\PlatformIO\Projects\Hexapod v3\Design\Mechanical Design\Kinematics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A94399-F0F9-444D-B350-275B96F5405C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F774419-B06F-4706-9248-32F96172EE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80FB6A6E-4815-48DC-A8C5-309DA8648198}"/>
   </bookViews>
   <sheets>
     <sheet name="X" sheetId="1" r:id="rId1"/>
@@ -538,22 +538,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>182.41</c:v>
+                  <c:v>199.32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-52.5</c:v>
+                  <c:v>-41.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-287.41000000000003</c:v>
+                  <c:v>-281.82</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-287.41000000000003</c:v>
+                  <c:v>-281.82</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-52.5</c:v>
+                  <c:v>-41.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>182.41</c:v>
+                  <c:v>199.32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -565,22 +565,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>135.63</c:v>
+                  <c:v>138.88999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>271.26</c:v>
+                  <c:v>277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>135.63</c:v>
+                  <c:v>138.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-271.26</c:v>
+                  <c:v>-277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -627,22 +627,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>287.41000000000003</c:v>
+                  <c:v>281.82</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>52.5</c:v>
+                  <c:v>41.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-182.41</c:v>
+                  <c:v>-199.32</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-182.41</c:v>
+                  <c:v>-199.32</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>52.5</c:v>
+                  <c:v>41.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>287.41000000000003</c:v>
+                  <c:v>281.82</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -654,22 +654,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>135.63</c:v>
+                  <c:v>138.88999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>271.26</c:v>
+                  <c:v>277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>135.63</c:v>
+                  <c:v>138.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-271.26</c:v>
+                  <c:v>-277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -716,22 +716,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>234.91</c:v>
+                  <c:v>240.57</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-234.91</c:v>
+                  <c:v>-240.57</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-234.91</c:v>
+                  <c:v>-240.57</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>234.91</c:v>
+                  <c:v>240.57</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -743,22 +743,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>135.63</c:v>
+                  <c:v>138.88999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>271.26</c:v>
+                  <c:v>277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>135.63</c:v>
+                  <c:v>138.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-271.26</c:v>
+                  <c:v>-277.79000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-135.63</c:v>
+                  <c:v>-138.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -26484,31 +26484,31 @@
         <v>0</v>
       </c>
       <c r="B5">
-        <v>182.41</v>
+        <v>199.32</v>
       </c>
       <c r="C5">
-        <v>135.63</v>
+        <v>138.88999999999999</v>
       </c>
       <c r="D5">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E5">
-        <v>287.41000000000003</v>
+        <v>281.82</v>
       </c>
       <c r="F5">
-        <v>135.63</v>
+        <v>138.88999999999999</v>
       </c>
       <c r="G5">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H5">
-        <v>234.91</v>
+        <v>240.57</v>
       </c>
       <c r="I5">
-        <v>135.63</v>
+        <v>138.88999999999999</v>
       </c>
       <c r="J5">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -26516,31 +26516,31 @@
         <v>1</v>
       </c>
       <c r="B6">
-        <v>-52.5</v>
+        <v>-41.25</v>
       </c>
       <c r="C6">
-        <v>271.26</v>
+        <v>277.79000000000002</v>
       </c>
       <c r="D6">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E6">
-        <v>52.5</v>
+        <v>41.25</v>
       </c>
       <c r="F6">
-        <v>271.26</v>
+        <v>277.79000000000002</v>
       </c>
       <c r="G6">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>271.26</v>
+        <v>277.79000000000002</v>
       </c>
       <c r="J6">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -26548,31 +26548,31 @@
         <v>2</v>
       </c>
       <c r="B7">
-        <v>-287.41000000000003</v>
+        <v>-281.82</v>
       </c>
       <c r="C7">
-        <v>135.63</v>
+        <v>138.9</v>
       </c>
       <c r="D7">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E7">
-        <v>-182.41</v>
+        <v>-199.32</v>
       </c>
       <c r="F7">
-        <v>135.63</v>
+        <v>138.9</v>
       </c>
       <c r="G7">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H7">
-        <v>-234.91</v>
+        <v>-240.57</v>
       </c>
       <c r="I7">
-        <v>135.63</v>
+        <v>138.9</v>
       </c>
       <c r="J7">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -26580,31 +26580,31 @@
         <v>3</v>
       </c>
       <c r="B8">
-        <v>-287.41000000000003</v>
+        <v>-281.82</v>
       </c>
       <c r="C8">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="D8">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E8">
-        <v>-182.41</v>
+        <v>-199.32</v>
       </c>
       <c r="F8">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="G8">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H8">
-        <v>-234.91</v>
+        <v>-240.57</v>
       </c>
       <c r="I8">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="J8">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -26612,31 +26612,31 @@
         <v>4</v>
       </c>
       <c r="B9">
-        <v>-52.5</v>
+        <v>-41.25</v>
       </c>
       <c r="C9">
-        <v>-271.26</v>
+        <v>-277.79000000000002</v>
       </c>
       <c r="D9">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E9">
-        <v>52.5</v>
+        <v>41.25</v>
       </c>
       <c r="F9">
-        <v>-271.26</v>
+        <v>-277.79000000000002</v>
       </c>
       <c r="G9">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>-271.26</v>
+        <v>-277.79000000000002</v>
       </c>
       <c r="J9">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -26644,31 +26644,31 @@
         <v>5</v>
       </c>
       <c r="B10">
-        <v>182.41</v>
+        <v>199.32</v>
       </c>
       <c r="C10">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="D10">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="E10">
-        <v>287.41000000000003</v>
+        <v>281.82</v>
       </c>
       <c r="F10">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="G10">
-        <v>-63.63</v>
+        <v>-89.66</v>
       </c>
       <c r="H10">
-        <v>234.91</v>
+        <v>240.57</v>
       </c>
       <c r="I10">
-        <v>-135.63</v>
+        <v>-138.9</v>
       </c>
       <c r="J10">
-        <v>-8.6300000000000008</v>
+        <v>-34.659999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>